<commit_message>
chore: toggle-slot via site
</commit_message>
<xml_diff>
--- a/STUDY PLAN 2026.xlsx
+++ b/STUDY PLAN 2026.xlsx
@@ -4451,7 +4451,11 @@
           <t>ALEMÃO</t>
         </is>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="4" t="n"/>

</xml_diff>

<commit_message>
chore: add-event via site
</commit_message>
<xml_diff>
--- a/STUDY PLAN 2026.xlsx
+++ b/STUDY PLAN 2026.xlsx
@@ -11,6 +11,7 @@
     <sheet name="OUTUBRO" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="NOVEMBRO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DEZEMBRO" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="EVENTS" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -9775,4 +9776,68 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>color</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mu8l4aa2sywv</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Geh</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>#FFD1DC</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: delete-event via site
</commit_message>
<xml_diff>
--- a/STUDY PLAN 2026.xlsx
+++ b/STUDY PLAN 2026.xlsx
@@ -9784,7 +9784,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9836,29 +9836,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>mu8l4mjcoe7r</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-09-19</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Gio</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>#C1FFF1</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: set-slot via site
</commit_message>
<xml_diff>
--- a/STUDY PLAN 2026.xlsx
+++ b/STUDY PLAN 2026.xlsx
@@ -4431,8 +4431,16 @@
           <t>NOT DONE</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="8" t="n"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>LIBRAS</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>NOT DONE</t>
+        </is>
+      </c>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="4" t="n"/>

</xml_diff>

<commit_message>
chore: log-session via site
</commit_message>
<xml_diff>
--- a/STUDY PLAN 2026.xlsx
+++ b/STUDY PLAN 2026.xlsx
@@ -12,6 +12,7 @@
     <sheet name="NOVEMBRO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="DEZEMBRO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="EVENTS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="POMODORO LOG" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -9825,4 +9826,60 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>timestamp</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>minutes</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>subject</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-21T22:50:34.570Z</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>30</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JAPONÊS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ciclo de foco concluído</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>